<commit_message>
Upload XLSX/XLS for Tests
</commit_message>
<xml_diff>
--- a/docs/test-template.xlsx
+++ b/docs/test-template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t xml:space="preserve">Sl. no</t>
   </si>
@@ -39,7 +39,10 @@
     <t xml:space="preserve">ANS key</t>
   </si>
   <si>
-    <t>POINT</t>
+    <t xml:space="preserve">Point (Optional)</t>
+  </si>
+  <si>
+    <t>Explanation(Optional)</t>
   </si>
   <si>
     <t xml:space="preserve">What is the least number divisible by 10,18,25</t>
@@ -91,7 +94,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -99,21 +102,27 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14.000000"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
     </font>
     <font>
-      <sz val="14.000000"/>
+      <sz val="12.000000"/>
       <name val="Times New Roman"/>
     </font>
     <font>
-      <sz val="14.000000"/>
+      <sz val="12.000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12.000000"/>
       <color indexed="64"/>
       <name val="Times New Roman"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -126,8 +135,14 @@
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor theme="8" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -135,32 +150,58 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="2" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf fontId="3" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -666,6 +707,7 @@
     <col bestFit="1" min="5" max="5" width="10.04296875"/>
     <col bestFit="1" min="6" max="6" width="10.33203125"/>
     <col bestFit="1" customWidth="1" min="7" max="7" width="10.5234375"/>
+    <col bestFit="1" min="9" max="9" width="19.28125"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25">
@@ -693,136 +735,309 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2" ht="17.25">
-      <c r="A2" s="4">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="6">
+        <v>350</v>
+      </c>
+      <c r="D2" s="6">
+        <v>450</v>
+      </c>
+      <c r="E2" s="6">
+        <v>320</v>
+      </c>
+      <c r="F2" s="6">
+        <v>500</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="6">
+        <v>1</v>
+      </c>
+      <c r="I2" s="7"/>
+    </row>
+    <row r="3" ht="17.25">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="8">
         <v>8</v>
       </c>
-      <c r="C2" s="5">
-        <v>350</v>
-      </c>
-      <c r="D2" s="5">
-        <v>450</v>
-      </c>
-      <c r="E2" s="5">
-        <v>320</v>
-      </c>
-      <c r="F2" s="5">
-        <v>500</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" s="5">
+      <c r="D3" s="8">
+        <v>11</v>
+      </c>
+      <c r="E3" s="8">
+        <v>13</v>
+      </c>
+      <c r="F3" s="6">
+        <v>17</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" ht="17.25">
-      <c r="A3" s="4">
-        <v>2</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="I3" s="7"/>
+    </row>
+    <row r="4" ht="17.25">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="6">
+        <v>16</v>
+      </c>
+      <c r="D4" s="6">
+        <v>22</v>
+      </c>
+      <c r="E4" s="6">
+        <v>30</v>
+      </c>
+      <c r="F4" s="6">
+        <v>35</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="6">
-        <v>8</v>
-      </c>
-      <c r="D3" s="6">
-        <v>11</v>
-      </c>
-      <c r="E3" s="6">
-        <v>13</v>
-      </c>
-      <c r="F3" s="5">
+      <c r="H4" s="6">
+        <v>1</v>
+      </c>
+      <c r="I4" s="7"/>
+    </row>
+    <row r="5" ht="17.25">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="5">
+      <c r="F5" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" ht="17.25">
-      <c r="A4" s="4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="5">
-        <v>16</v>
-      </c>
-      <c r="D4" s="5">
+      <c r="I5" s="7"/>
+    </row>
+    <row r="6" ht="17.25">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="5">
-        <v>30</v>
-      </c>
-      <c r="F4" s="5">
-        <v>35</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H4" s="5">
+      <c r="F6" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" ht="17.25">
-      <c r="A5" s="4">
-        <v>4</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" ht="17.25">
-      <c r="A6" s="4">
-        <v>5</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H6" s="5">
-        <v>1</v>
-      </c>
+      <c r="I6" s="7"/>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="A10" s="11"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" ht="14.25">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>